<commit_message>
NEW: STALL QR PRINTING,1. PRINT,2. REPORT,3. IMPORT,4. SETTINGS
</commit_message>
<xml_diff>
--- a/Business_Process_Master_List.xlsx
+++ b/Business_Process_Master_List.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V18"/>
+  <dimension ref="A1:V24"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -570,7 +570,7 @@
         <v>Interview Feedback Capture</v>
       </c>
       <c r="D3" t="str">
-        <v>Public form capturing candidate name, mobile number, designation, department, address, 10 rating questions (EN/TA bilingual), referral flag and free-text comments.</v>
+        <v>Public form capturing candidate name, mobile number, designation, department, interview location, address, 10 rating questions (EN/TA bilingual), referral flag and free-text comments.</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -638,7 +638,7 @@
         <v>Rating Input Control</v>
       </c>
       <c r="D4" t="str">
-        <v>Reusable 1-5 star/scale rating UI used across the 10 feedback questions.</v>
+        <v>Reusable 1-5 star/scale rating UI used across the 10 feedback questions; shows red border and inline bilingual (EN/TA) "Please select a rating" message when left unanswered (error prop, v2.6.0).</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -771,22 +771,22 @@
         <v>HR Interview Feedback &amp; Quiz Portal</v>
       </c>
       <c r="C6" t="str">
-        <v>QR Code Display</v>
+        <v>Interview Location Capture</v>
       </c>
       <c r="D6" t="str">
-        <v>Generates a scannable QR code (qrcode.react) linking to the feedback form for candidates to open on their own device.</v>
+        <v>Required Interview Location dropdown (Attayampalayam, Thindal, Vilarasampatti) from BRANCHES master in constants.ts; stored in hrfeedbacks.branch (v2.6.0).</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" t="str">
-        <v>QR Code</v>
+        <v>Feedback Form</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H6" t="str">
-        <v>Transaction</v>
+        <v>Master</v>
       </c>
       <c r="I6" t="str">
         <v>No</v>
@@ -804,7 +804,7 @@
         <v>HR Team</v>
       </c>
       <c r="N6" t="str">
-        <v>Candidate</v>
+        <v>HR Team</v>
       </c>
       <c r="O6" t="str">
         <v>No</v>
@@ -813,22 +813,22 @@
         <v>No</v>
       </c>
       <c r="Q6" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R6" t="str">
-        <v>—</v>
+        <v>Branch list hardcoded in frontend constants; adding a location needs a code change and redeploy</v>
       </c>
       <c r="S6" t="str">
-        <v>—</v>
+        <v>2026-10-16</v>
       </c>
       <c r="T6" t="str">
-        <v>—</v>
+        <v>Move branch list to a DB master table maintained by HR</v>
       </c>
       <c r="U6" t="str">
         <v>—</v>
       </c>
       <c r="V6" t="str">
-        <v>—</v>
+        <v>Developer</v>
       </c>
     </row>
     <row r="7">
@@ -839,19 +839,19 @@
         <v>HR Interview Feedback &amp; Quiz Portal</v>
       </c>
       <c r="C7" t="str">
-        <v>HR Login</v>
+        <v>Required-Field Validation</v>
       </c>
       <c r="D7" t="str">
-        <v>Username/password gate that unlocks Admin Dashboard and Quiz Manager views.</v>
+        <v>On submit, validates Candidate Name, Mobile, Designation, Department, Interview Location, Address, all 10 ratings and referral Yes/No; highlights missing fields in red with inline EN/TA errors and a summary banner; errors clear live as fields are corrected (v2.6.0).</v>
       </c>
       <c r="E7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F7" t="str">
-        <v>Authentication</v>
+        <v>Feedback Form</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H7" t="str">
         <v>Transaction</v>
@@ -866,13 +866,13 @@
         <v>Developer</v>
       </c>
       <c r="L7" t="str">
-        <v>IT Lead</v>
+        <v>HR Lead</v>
       </c>
       <c r="M7" t="str">
-        <v>HR Lead</v>
+        <v>HR Team</v>
       </c>
       <c r="N7" t="str">
-        <v>HR Team</v>
+        <v>Candidate</v>
       </c>
       <c r="O7" t="str">
         <v>No</v>
@@ -884,13 +884,13 @@
         <v>Yes</v>
       </c>
       <c r="R7" t="str">
-        <v>Credentials are hardcoded in frontend source (LoginForm.tsx) with no hashing/session/token; client-side only gate</v>
+        <v>Validation is client-side only; POST /api/feedback accepts records with missing fields (e.g. null branch)</v>
       </c>
       <c r="S7" t="str">
-        <v>2026-08-20</v>
+        <v>2026-10-16</v>
       </c>
       <c r="T7" t="str">
-        <v>Move auth to backend with hashed credentials + session/JWT; remove hardcoded creds from source</v>
+        <v>Mirror required-field checks in server.js and reject incomplete payloads with 400</v>
       </c>
       <c r="U7" t="str">
         <v>—</v>
@@ -907,16 +907,16 @@
         <v>HR Interview Feedback &amp; Quiz Portal</v>
       </c>
       <c r="C8" t="str">
-        <v>Feedback Analytics Dashboard</v>
+        <v>QR Code Display</v>
       </c>
       <c r="D8" t="str">
-        <v>Admin view of all submitted feedback with aggregated ratings, filters and drill-down per candidate.</v>
+        <v>Generates a scannable QR code (qrcode.react) linking to the feedback form for candidates to open on their own device.</v>
       </c>
       <c r="E8">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F8" t="str">
-        <v>Admin Dashboard</v>
+        <v>QR Code</v>
       </c>
       <c r="G8">
         <v>1</v>
@@ -925,7 +925,7 @@
         <v>Transaction</v>
       </c>
       <c r="I8" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="J8" t="str">
         <v>Yes</v>
@@ -934,37 +934,37 @@
         <v>Developer</v>
       </c>
       <c r="L8" t="str">
-        <v>IT Lead</v>
+        <v>HR Lead</v>
       </c>
       <c r="M8" t="str">
-        <v>HR Lead</v>
+        <v>HR Team</v>
       </c>
       <c r="N8" t="str">
-        <v>HR Team</v>
+        <v>Candidate</v>
       </c>
       <c r="O8" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="P8" t="str">
         <v>No</v>
       </c>
       <c r="Q8" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="R8" t="str">
-        <v>Dashboard route guarded only by client-side isLoggedIn state, not server-verified session</v>
+        <v>—</v>
       </c>
       <c r="S8" t="str">
-        <v>2026-08-20</v>
+        <v>—</v>
       </c>
       <c r="T8" t="str">
-        <v>Enforce server-side auth/session check on all /api endpoints, not just UI routing</v>
+        <v>—</v>
       </c>
       <c r="U8" t="str">
         <v>—</v>
       </c>
       <c r="V8" t="str">
-        <v>Developer</v>
+        <v>—</v>
       </c>
     </row>
     <row r="9">
@@ -975,19 +975,19 @@
         <v>HR Interview Feedback &amp; Quiz Portal</v>
       </c>
       <c r="C9" t="str">
-        <v>AI Feedback Analysis</v>
+        <v>HR Login</v>
       </c>
       <c r="D9" t="str">
-        <v>Sends feedback dataset to Google Gemini API to generate summary, strengths, weaknesses, recommendations and sentiment score.</v>
+        <v>Username/password gate that unlocks Admin Dashboard and Quiz Manager views.</v>
       </c>
       <c r="E9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F9" t="str">
-        <v>Admin Dashboard</v>
+        <v>Authentication</v>
       </c>
       <c r="G9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H9" t="str">
         <v>Transaction</v>
@@ -1011,7 +1011,7 @@
         <v>HR Team</v>
       </c>
       <c r="O9" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="P9" t="str">
         <v>No</v>
@@ -1020,13 +1020,13 @@
         <v>Yes</v>
       </c>
       <c r="R9" t="str">
-        <v>Candidate PII (name, mobile, address, comments) sent to third-party Gemini API in full</v>
+        <v>Credentials are hardcoded in frontend source (LoginForm.tsx) with no hashing/session/token; client-side only gate</v>
       </c>
       <c r="S9" t="str">
         <v>2026-08-20</v>
       </c>
       <c r="T9" t="str">
-        <v>Strip/mask PII before sending to external AI service; review Gemini data-retention terms</v>
+        <v>Move auth to backend with hashed credentials + session/JWT; remove hardcoded creds from source</v>
       </c>
       <c r="U9" t="str">
         <v>—</v>
@@ -1043,10 +1043,10 @@
         <v>HR Interview Feedback &amp; Quiz Portal</v>
       </c>
       <c r="C10" t="str">
-        <v>Feedback Excel Export</v>
+        <v>Feedback Analytics Dashboard</v>
       </c>
       <c r="D10" t="str">
-        <v>Exports all feedback records (incl. PII) to a downloadable .xlsx file via SheetJS.</v>
+        <v>Admin view of all submitted feedback with aggregated ratings, filters and drill-down per candidate; entry list and detail modal show Designation, Department and Interview Location.</v>
       </c>
       <c r="E10">
         <v>4</v>
@@ -1055,7 +1055,7 @@
         <v>Admin Dashboard</v>
       </c>
       <c r="G10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H10" t="str">
         <v>Transaction</v>
@@ -1088,13 +1088,13 @@
         <v>Yes</v>
       </c>
       <c r="R10" t="str">
-        <v>Unrestricted export of PII to local file with no audit trail of who exported/when</v>
+        <v>Dashboard route guarded only by client-side isLoggedIn state, not server-verified session</v>
       </c>
       <c r="S10" t="str">
         <v>2026-08-20</v>
       </c>
       <c r="T10" t="str">
-        <v>Add export audit logging; consider redacting mobile numbers in export</v>
+        <v>Enforce server-side auth/session check on all /api endpoints, not just UI routing</v>
       </c>
       <c r="U10" t="str">
         <v>—</v>
@@ -1111,25 +1111,25 @@
         <v>HR Interview Feedback &amp; Quiz Portal</v>
       </c>
       <c r="C11" t="str">
-        <v>Quiz Contest</v>
+        <v>AI Feedback Analysis</v>
       </c>
       <c r="D11" t="str">
-        <v>Timed candidate quiz supporting Multiple Choice, Picture Choice, Memory Test and Jumbled Word question types, scored per active question set.</v>
+        <v>Sends feedback dataset to Google Gemini API to generate summary, strengths, weaknesses, recommendations and sentiment score.</v>
       </c>
       <c r="E11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F11" t="str">
-        <v>Quiz Contest</v>
+        <v>Admin Dashboard</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H11" t="str">
         <v>Transaction</v>
       </c>
       <c r="I11" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="J11" t="str">
         <v>Yes</v>
@@ -1138,13 +1138,13 @@
         <v>Developer</v>
       </c>
       <c r="L11" t="str">
+        <v>IT Lead</v>
+      </c>
+      <c r="M11" t="str">
         <v>HR Lead</v>
       </c>
-      <c r="M11" t="str">
-        <v>HR Team</v>
-      </c>
       <c r="N11" t="str">
-        <v>Candidate</v>
+        <v>HR Team</v>
       </c>
       <c r="O11" t="str">
         <v>Yes</v>
@@ -1153,22 +1153,22 @@
         <v>No</v>
       </c>
       <c r="Q11" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R11" t="str">
-        <v>—</v>
+        <v>Candidate PII (name, mobile, address, comments) sent to third-party Gemini API in full</v>
       </c>
       <c r="S11" t="str">
-        <v>—</v>
+        <v>2026-08-20</v>
       </c>
       <c r="T11" t="str">
-        <v>—</v>
+        <v>Strip/mask PII before sending to external AI service; review Gemini data-retention terms</v>
       </c>
       <c r="U11" t="str">
         <v>—</v>
       </c>
       <c r="V11" t="str">
-        <v>—</v>
+        <v>Developer</v>
       </c>
     </row>
     <row r="12">
@@ -1179,25 +1179,25 @@
         <v>HR Interview Feedback &amp; Quiz Portal</v>
       </c>
       <c r="C12" t="str">
-        <v>Quiz Result Submission</v>
+        <v>Feedback Excel Export</v>
       </c>
       <c r="D12" t="str">
-        <v>Submits candidate quiz score/result to backend (hrquiz_results); falls back to local state if API call fails.</v>
+        <v>Exports all feedback records (incl. PII and Interview Location column) to a downloadable .xlsx file via SheetJS.</v>
       </c>
       <c r="E12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F12" t="str">
-        <v>Quiz Contest</v>
+        <v>Admin Dashboard</v>
       </c>
       <c r="G12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H12" t="str">
         <v>Transaction</v>
       </c>
       <c r="I12" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="J12" t="str">
         <v>Yes</v>
@@ -1206,11 +1206,11 @@
         <v>Developer</v>
       </c>
       <c r="L12" t="str">
+        <v>IT Lead</v>
+      </c>
+      <c r="M12" t="str">
         <v>HR Lead</v>
       </c>
-      <c r="M12" t="str">
-        <v>IT Team</v>
-      </c>
       <c r="N12" t="str">
         <v>HR Team</v>
       </c>
@@ -1221,22 +1221,22 @@
         <v>No</v>
       </c>
       <c r="Q12" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R12" t="str">
-        <v>—</v>
+        <v>Unrestricted export of PII to local file with no audit trail of who exported/when</v>
       </c>
       <c r="S12" t="str">
-        <v>—</v>
+        <v>2026-08-20</v>
       </c>
       <c r="T12" t="str">
-        <v>—</v>
+        <v>Add export audit logging; consider redacting mobile numbers in export</v>
       </c>
       <c r="U12" t="str">
         <v>—</v>
       </c>
       <c r="V12" t="str">
-        <v>—</v>
+        <v>Developer</v>
       </c>
     </row>
     <row r="13">
@@ -1247,16 +1247,16 @@
         <v>HR Interview Feedback &amp; Quiz Portal</v>
       </c>
       <c r="C13" t="str">
-        <v>Live Leaderboard</v>
+        <v>Quiz Contest</v>
       </c>
       <c r="D13" t="str">
-        <v>Displays ranked quiz results filtered by active/enabled question sets, with set switcher.</v>
+        <v>Timed candidate quiz supporting Multiple Choice, Picture Choice, Memory Test and Jumbled Word question types, scored per active question set.</v>
       </c>
       <c r="E13">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F13" t="str">
-        <v>Live Results</v>
+        <v>Quiz Contest</v>
       </c>
       <c r="G13">
         <v>1</v>
@@ -1292,19 +1292,19 @@
         <v>No</v>
       </c>
       <c r="R13" t="str">
-        <v>Leaderboard shows candidate name/mobile publicly with no consent gate</v>
+        <v>—</v>
       </c>
       <c r="S13" t="str">
-        <v>2026-08-20</v>
+        <v>—</v>
       </c>
       <c r="T13" t="str">
-        <v>Add explicit consent/opt-out for public display of name &amp; mobile on leaderboard</v>
+        <v>—</v>
       </c>
       <c r="U13" t="str">
         <v>—</v>
       </c>
       <c r="V13" t="str">
-        <v>Developer</v>
+        <v>—</v>
       </c>
     </row>
     <row r="14">
@@ -1315,25 +1315,25 @@
         <v>HR Interview Feedback &amp; Quiz Portal</v>
       </c>
       <c r="C14" t="str">
-        <v>Quiz Question Management</v>
+        <v>Quiz Result Submission</v>
       </c>
       <c r="D14" t="str">
-        <v>Admin CRUD for quiz questions (create/edit/delete, question type, options, correct answer, active flag, sort order, set assignment).</v>
+        <v>Submits candidate quiz score/result to backend (hrquiz_results); falls back to local state if API call fails.</v>
       </c>
       <c r="E14">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F14" t="str">
-        <v>Quiz Manager</v>
+        <v>Quiz Contest</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H14" t="str">
-        <v>Master</v>
+        <v>Transaction</v>
       </c>
       <c r="I14" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="J14" t="str">
         <v>Yes</v>
@@ -1342,22 +1342,22 @@
         <v>Developer</v>
       </c>
       <c r="L14" t="str">
-        <v>IT Lead</v>
+        <v>HR Lead</v>
       </c>
       <c r="M14" t="str">
-        <v>HR Lead</v>
+        <v>IT Team</v>
       </c>
       <c r="N14" t="str">
         <v>HR Team</v>
       </c>
       <c r="O14" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="P14" t="str">
         <v>No</v>
       </c>
       <c r="Q14" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="R14" t="str">
         <v>—</v>
@@ -1383,22 +1383,22 @@
         <v>HR Interview Feedback &amp; Quiz Portal</v>
       </c>
       <c r="C15" t="str">
-        <v>Quiz Question Bulk Import</v>
+        <v>Live Leaderboard</v>
       </c>
       <c r="D15" t="str">
-        <v>Imports question sets in bulk from an uploaded Excel workbook (one sheet per set) via SheetJS parser.</v>
+        <v>Displays ranked quiz results filtered by active/enabled question sets, with set switcher.</v>
       </c>
       <c r="E15">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F15" t="str">
-        <v>Quiz Manager</v>
+        <v>Live Results</v>
       </c>
       <c r="G15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H15" t="str">
-        <v>Master</v>
+        <v>Transaction</v>
       </c>
       <c r="I15" t="str">
         <v>No</v>
@@ -1410,31 +1410,31 @@
         <v>Developer</v>
       </c>
       <c r="L15" t="str">
-        <v>IT Lead</v>
+        <v>HR Lead</v>
       </c>
       <c r="M15" t="str">
-        <v>HR Lead</v>
+        <v>HR Team</v>
       </c>
       <c r="N15" t="str">
-        <v>—</v>
+        <v>Candidate</v>
       </c>
       <c r="O15" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="P15" t="str">
         <v>No</v>
       </c>
       <c r="Q15" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="R15" t="str">
-        <v>No schema/type validation shown on imported rows beyond basic mapping</v>
+        <v>Leaderboard shows candidate name/mobile publicly with no consent gate</v>
       </c>
       <c r="S15" t="str">
         <v>2026-08-20</v>
       </c>
       <c r="T15" t="str">
-        <v>Validate imported rows (required fields, answer format) before commit</v>
+        <v>Add explicit consent/opt-out for public display of name &amp; mobile on leaderboard</v>
       </c>
       <c r="U15" t="str">
         <v>—</v>
@@ -1451,10 +1451,10 @@
         <v>HR Interview Feedback &amp; Quiz Portal</v>
       </c>
       <c r="C16" t="str">
-        <v>Quiz Settings Control</v>
+        <v>Quiz Question Management</v>
       </c>
       <c r="D16" t="str">
-        <v>Toggles quiz active/inactive, sets per-question timer, active question set and enabled sets list.</v>
+        <v>Admin CRUD for quiz questions (create/edit/delete, question type, options, correct answer, active flag, sort order, set assignment).</v>
       </c>
       <c r="E16">
         <v>7</v>
@@ -1463,7 +1463,7 @@
         <v>Quiz Manager</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H16" t="str">
         <v>Master</v>
@@ -1519,25 +1519,25 @@
         <v>HR Interview Feedback &amp; Quiz Portal</v>
       </c>
       <c r="C17" t="str">
-        <v>Feedback &amp; Quiz REST API</v>
+        <v>Quiz Question Bulk Import</v>
       </c>
       <c r="D17" t="str">
-        <v>Express API (server.js) exposing /api/feedback and /api/quiz/* endpoints backed by MSSQL; auto-creates schema (hrfeedbacks, hrquiz_questions, hrquiz_settings, hrquiz_results) on boot.</v>
+        <v>Imports question sets in bulk from an uploaded Excel workbook (one sheet per set) via SheetJS parser.</v>
       </c>
       <c r="E17">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F17" t="str">
-        <v>Backend API</v>
+        <v>Quiz Manager</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H17" t="str">
-        <v>Transaction</v>
+        <v>Master</v>
       </c>
       <c r="I17" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="J17" t="str">
         <v>Yes</v>
@@ -1549,13 +1549,13 @@
         <v>IT Lead</v>
       </c>
       <c r="M17" t="str">
-        <v>IT Team</v>
+        <v>HR Lead</v>
       </c>
       <c r="N17" t="str">
-        <v>HR Team</v>
+        <v>—</v>
       </c>
       <c r="O17" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="P17" t="str">
         <v>No</v>
@@ -1564,13 +1564,13 @@
         <v>Yes</v>
       </c>
       <c r="R17" t="str">
-        <v>No authentication/authorization on any API route — all endpoints (read &amp; write) are publicly callable</v>
+        <v>No schema/type validation shown on imported rows beyond basic mapping</v>
       </c>
       <c r="S17" t="str">
         <v>2026-08-20</v>
       </c>
       <c r="T17" t="str">
-        <v>Add API auth (session/JWT/API key) at least on write endpoints and admin-only reads</v>
+        <v>Validate imported rows (required fields, answer format) before commit</v>
       </c>
       <c r="U17" t="str">
         <v>—</v>
@@ -1587,19 +1587,19 @@
         <v>HR Interview Feedback &amp; Quiz Portal</v>
       </c>
       <c r="C18" t="str">
-        <v>Database Connectivity</v>
+        <v>Quiz Settings Control</v>
       </c>
       <c r="D18" t="str">
-        <v>MSSQL connection pool (mssql driver) configured via .env (DB_USER/PASSWORD/SERVER/DATABASE); encrypt disabled, trustServerCertificate on.</v>
+        <v>Toggles quiz active/inactive, sets per-question timer, active question set and enabled sets list.</v>
       </c>
       <c r="E18">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F18" t="str">
-        <v>Backend API</v>
+        <v>Quiz Manager</v>
       </c>
       <c r="G18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H18" t="str">
         <v>Master</v>
@@ -1617,39 +1617,447 @@
         <v>IT Lead</v>
       </c>
       <c r="M18" t="str">
+        <v>HR Lead</v>
+      </c>
+      <c r="N18" t="str">
+        <v>HR Team</v>
+      </c>
+      <c r="O18" t="str">
+        <v>No</v>
+      </c>
+      <c r="P18" t="str">
+        <v>No</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="R18" t="str">
+        <v>—</v>
+      </c>
+      <c r="S18" t="str">
+        <v>—</v>
+      </c>
+      <c r="T18" t="str">
+        <v>—</v>
+      </c>
+      <c r="U18" t="str">
+        <v>—</v>
+      </c>
+      <c r="V18" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>HR Interview Feedback &amp; Quiz Portal</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Feedback &amp; Quiz REST API</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Express API (server.js) exposing /api/feedback and /api/quiz/* endpoints backed by MSSQL; auto-creates schema (hrfeedbacks, hrquiz_questions, hrquiz_settings, hrquiz_results) on boot and auto-migrates the hrfeedbacks.branch (Interview Location) column for existing databases.</v>
+      </c>
+      <c r="E19">
+        <v>8</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Backend API</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Transaction</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="L19" t="str">
+        <v>IT Lead</v>
+      </c>
+      <c r="M19" t="str">
         <v>IT Team</v>
       </c>
-      <c r="N18" t="str">
-        <v>—</v>
-      </c>
-      <c r="O18" t="str">
-        <v>No</v>
-      </c>
-      <c r="P18" t="str">
-        <v>No</v>
-      </c>
-      <c r="Q18" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="R18" t="str">
+      <c r="N19" t="str">
+        <v>HR Team</v>
+      </c>
+      <c r="O19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="P19" t="str">
+        <v>No</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="R19" t="str">
+        <v>No authentication/authorization on any API route — all endpoints (read &amp; write) are publicly callable</v>
+      </c>
+      <c r="S19" t="str">
+        <v>2026-08-20</v>
+      </c>
+      <c r="T19" t="str">
+        <v>Add API auth (session/JWT/API key) at least on write endpoints and admin-only reads</v>
+      </c>
+      <c r="U19" t="str">
+        <v>—</v>
+      </c>
+      <c r="V19" t="str">
+        <v>Developer</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>HR Interview Feedback &amp; Quiz Portal</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Database Connectivity</v>
+      </c>
+      <c r="D20" t="str">
+        <v>MSSQL connection pool (mssql driver) configured via .env (DB_USER/PASSWORD/SERVER/DATABASE); encrypt disabled, trustServerCertificate on.</v>
+      </c>
+      <c r="E20">
+        <v>8</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Backend API</v>
+      </c>
+      <c r="G20">
+        <v>2</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Master</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="L20" t="str">
+        <v>IT Lead</v>
+      </c>
+      <c r="M20" t="str">
+        <v>IT Team</v>
+      </c>
+      <c r="N20" t="str">
+        <v>—</v>
+      </c>
+      <c r="O20" t="str">
+        <v>No</v>
+      </c>
+      <c r="P20" t="str">
+        <v>No</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="R20" t="str">
         <v>DB traffic encryption disabled (encrypt:false) and TLS cert trust bypassed</v>
       </c>
-      <c r="S18" t="str">
+      <c r="S20" t="str">
         <v>2026-08-20</v>
       </c>
-      <c r="T18" t="str">
+      <c r="T20" t="str">
         <v>Enable encrypt:true with a valid certificate for production DB connections</v>
       </c>
-      <c r="U18" t="str">
-        <v>—</v>
-      </c>
-      <c r="V18" t="str">
+      <c r="U20" t="str">
+        <v>—</v>
+      </c>
+      <c r="V20" t="str">
         <v>IT Team</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>HR Interview Feedback &amp; Quiz Portal</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Stall QR Coupon Print</v>
+      </c>
+      <c r="D21" t="str">
+        <v>HR enters/scans Employee ID; atomically marks employee printed in BBLive StallEmployeeMaster and prints 80mm slip with company address, QR (EmpCode|Name|Company|Dept|Amount|Date) and amount; repeat print blocked, explicit Reprint prints "REPRINT" slip and is logged in StallPrintLog (v2.7.0).</v>
+      </c>
+      <c r="E21">
+        <v>9</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Stall QR</v>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Transaction</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="L21" t="str">
+        <v>HR Lead</v>
+      </c>
+      <c r="M21" t="str">
+        <v>IT Team</v>
+      </c>
+      <c r="N21" t="str">
+        <v>HR Team</v>
+      </c>
+      <c r="O21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="P21" t="str">
+        <v>No</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="R21" t="str">
+        <v>Reprint allowed for any logged-in HR user with no approval step</v>
+      </c>
+      <c r="S21" t="str">
+        <v>2026-10-23</v>
+      </c>
+      <c r="T21" t="str">
+        <v>Add reprint reason / approver if misuse is observed</v>
+      </c>
+      <c r="U21" t="str">
+        <v>—</v>
+      </c>
+      <c r="V21" t="str">
+        <v>Developer</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>HR Interview Feedback &amp; Quiz Portal</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Stall Employee Import</v>
+      </c>
+      <c r="D22" t="str">
+        <v>HR uploads Excel (EmpCode, EmpName, Company, Department); client validates missing values, code format, duplicates and missing company addresses; server re-validates and deletes old data + inserts new rows in one transaction (v2.7.0).</v>
+      </c>
+      <c r="E22">
+        <v>9</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Stall QR</v>
+      </c>
+      <c r="G22">
+        <v>2</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Master</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="L22" t="str">
+        <v>HR Lead</v>
+      </c>
+      <c r="M22" t="str">
+        <v>IT Team</v>
+      </c>
+      <c r="N22" t="str">
+        <v>HR Team</v>
+      </c>
+      <c r="O22" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="P22" t="str">
+        <v>No</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="R22" t="str">
+        <v>Import wipes previous print status; history only kept in StallPrintLog for prints made via the portal</v>
+      </c>
+      <c r="S22" t="str">
+        <v>2026-10-23</v>
+      </c>
+      <c r="T22" t="str">
+        <v>Take a backup of StallEmployeeMaster before each import if old status is needed</v>
+      </c>
+      <c r="U22" t="str">
+        <v>—</v>
+      </c>
+      <c r="V22" t="str">
+        <v>HR Team</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>HR Interview Feedback &amp; Quiz Portal</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Stall Print Report</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Printed / pending / reprint counts with search, company and status filters, per-row Print/Reprint and Excel export (v2.7.0).</v>
+      </c>
+      <c r="E23">
+        <v>9</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Stall QR</v>
+      </c>
+      <c r="G23">
+        <v>3</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Transaction</v>
+      </c>
+      <c r="I23" t="str">
+        <v>No</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="L23" t="str">
+        <v>HR Lead</v>
+      </c>
+      <c r="M23" t="str">
+        <v>HR Team</v>
+      </c>
+      <c r="N23" t="str">
+        <v>HR Team</v>
+      </c>
+      <c r="O23" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="P23" t="str">
+        <v>No</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>No</v>
+      </c>
+      <c r="R23" t="str">
+        <v>—</v>
+      </c>
+      <c r="S23" t="str">
+        <v>—</v>
+      </c>
+      <c r="T23" t="str">
+        <v>—</v>
+      </c>
+      <c r="U23" t="str">
+        <v>—</v>
+      </c>
+      <c r="V23" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>HR Interview Feedback &amp; Quiz Portal</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Stall Settings</v>
+      </c>
+      <c r="D24" t="str">
+        <v>HR-maintained coupon amount (StallSettings) and per-company print address (StallCompanyAddress); reprints keep the amount of the original print (v2.7.0).</v>
+      </c>
+      <c r="E24">
+        <v>9</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Stall QR</v>
+      </c>
+      <c r="G24">
+        <v>4</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Master</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="L24" t="str">
+        <v>HR Lead</v>
+      </c>
+      <c r="M24" t="str">
+        <v>HR Team</v>
+      </c>
+      <c r="N24" t="str">
+        <v>HR Team</v>
+      </c>
+      <c r="O24" t="str">
+        <v>No</v>
+      </c>
+      <c r="P24" t="str">
+        <v>No</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="R24" t="str">
+        <v>Amount change has no audit trail of who changed it</v>
+      </c>
+      <c r="S24" t="str">
+        <v>2026-10-23</v>
+      </c>
+      <c r="T24" t="str">
+        <v>Log amount changes with user and timestamp</v>
+      </c>
+      <c r="U24" t="str">
+        <v>—</v>
+      </c>
+      <c r="V24" t="str">
+        <v>Developer</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>